<commit_message>
Änderung auf neuen Varaktor
</commit_message>
<xml_diff>
--- a/kicad/Wien-Bruecken-VCO_5MHz5/BOM_Wien-LT_TB.xlsx
+++ b/kicad/Wien-Bruecken-VCO_5MHz5/BOM_Wien-LT_TB.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\torbe\Documents\2.0 Studium\6.0 Semester\M6.10 Analoge Schaltungen (ANS)\ANS-VCO-Projekt-2026\kicad\Wien-Bruecken-VCO_5MHz5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/icke/Desktop/Git.nosync/ANS-VCO-Projekt-2026/kicad/Wien-Bruecken-VCO_5MHz5/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{396038E3-A73B-4720-9979-B2C51681B07D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F9A687E-5B2A-E14E-AA8B-8B4DF2D69395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="38400" windowHeight="24100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
         <sz val="10"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
-        <charset val="134"/>
+        <family val="2"/>
       </rPr>
       <t>*</t>
     </r>
@@ -50,7 +50,7 @@
         <b/>
         <sz val="10"/>
         <rFont val="Arial"/>
-        <charset val="134"/>
+        <family val="2"/>
       </rPr>
       <t>Designator</t>
     </r>
@@ -62,7 +62,7 @@
         <sz val="10"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
-        <charset val="134"/>
+        <family val="2"/>
       </rPr>
       <t>*</t>
     </r>
@@ -71,7 +71,7 @@
         <b/>
         <sz val="10"/>
         <rFont val="Arial"/>
-        <charset val="134"/>
+        <family val="2"/>
       </rPr>
       <t>Qty</t>
     </r>
@@ -86,7 +86,7 @@
         <sz val="10"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
-        <charset val="134"/>
+        <family val="2"/>
       </rPr>
       <t>*</t>
     </r>
@@ -95,7 +95,7 @@
         <b/>
         <sz val="10"/>
         <rFont val="Arial"/>
-        <charset val="134"/>
+        <family val="2"/>
       </rPr>
       <t>Mfg Part #</t>
     </r>
@@ -110,7 +110,7 @@
         <sz val="10"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
-        <charset val="134"/>
+        <family val="2"/>
       </rPr>
       <t>*</t>
     </r>
@@ -119,7 +119,7 @@
         <b/>
         <sz val="10"/>
         <rFont val="Arial"/>
-        <charset val="134"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Package/Footprint </t>
     </r>
@@ -188,21 +188,9 @@
     <t>Den wird es wohl schon geben im Labor</t>
   </si>
   <si>
-    <t>D2,D3,D4,D5,D6,D7,D8,D9</t>
-  </si>
-  <si>
     <t>Philips</t>
   </si>
   <si>
-    <t>BB909A</t>
-  </si>
-  <si>
-    <t>BB909A - Varicap-Diode, 30 V, 20 mA, 2,6 – 31 pF, DO-34</t>
-  </si>
-  <si>
-    <t>SO-34</t>
-  </si>
-  <si>
     <t>C…</t>
   </si>
   <si>
@@ -264,13 +252,25 @@
   </si>
   <si>
     <t>J113</t>
+  </si>
+  <si>
+    <t>D2,D3,D4</t>
+  </si>
+  <si>
+    <t>BB535</t>
+  </si>
+  <si>
+    <t>SOD-323</t>
+  </si>
+  <si>
+    <t>Infineon Technologies Kapazitätsdiode BB535 30 V 20 mA Einzeln SOD 323 Tape cut</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -281,7 +281,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -303,13 +303,13 @@
       <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -349,7 +349,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -371,6 +371,14 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -425,15 +433,9 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
@@ -495,10 +497,19 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Link" xfId="1" builtinId="8"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -761,415 +772,415 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:I26"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="9" style="3"/>
-    <col min="2" max="2" width="16.33203125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="9" style="3"/>
-    <col min="4" max="4" width="21.33203125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="29.796875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="41.6640625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="20.796875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="13.6640625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="35.6640625" style="3" customWidth="1"/>
-    <col min="10" max="16384" width="9" style="3"/>
+    <col min="1" max="1" width="9" style="1"/>
+    <col min="2" max="2" width="16.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9" style="1"/>
+    <col min="4" max="4" width="21.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29.83203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="41.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="35.6640625" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:9" ht="19.5" customHeight="1">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="D2" s="2" t="s">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="D2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
     </row>
     <row r="6" spans="1:9" ht="28.5" customHeight="1">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="14.25">
-      <c r="A7" s="7">
+    <row r="7" spans="1:9" ht="15">
+      <c r="A7" s="5">
         <v>1</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="5">
         <v>1</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="10"/>
-    </row>
-    <row r="8" spans="1:9" ht="14.25">
-      <c r="A8" s="7">
+      <c r="I7" s="8"/>
+    </row>
+    <row r="8" spans="1:9" ht="15">
+      <c r="A8" s="5">
         <v>2</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="5">
         <v>1</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10" t="s">
+      <c r="E8" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="10"/>
-    </row>
-    <row r="9" spans="1:9" ht="14.25">
-      <c r="A9" s="7">
+      <c r="I8" s="8"/>
+    </row>
+    <row r="9" spans="1:9" ht="15">
+      <c r="A9" s="5">
         <v>3</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="5">
         <v>1</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F9" s="10" t="s">
+      <c r="E9" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="10"/>
-    </row>
-    <row r="10" spans="1:9" ht="14.25">
-      <c r="A10" s="7">
+      <c r="I9" s="8"/>
+    </row>
+    <row r="10" spans="1:9" ht="15">
+      <c r="A10" s="5">
         <v>4</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="24">
+      <c r="C10" s="22">
         <v>0</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E10" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="I10" s="8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="14.25">
-      <c r="A11" s="7">
+    <row r="11" spans="1:9" ht="15">
+      <c r="A11" s="5">
         <v>5</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="5">
+        <v>4</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="7">
+      <c r="E11" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="8"/>
+    </row>
+    <row r="12" spans="1:9" ht="15">
+      <c r="A12" s="5">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="22">
+        <v>0</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="15">
+      <c r="A13" s="5">
+        <v>7</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="5">
+        <v>2</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="15">
+      <c r="A14" s="5">
         <v>8</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="I11" s="10"/>
-    </row>
-    <row r="12" spans="1:9" ht="14.25">
-      <c r="A12" s="7">
-        <v>6</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="24">
-        <v>0</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E12" t="s">
-        <v>36</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="I12" s="10" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="14.25">
-      <c r="A13" s="7">
-        <v>7</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="7">
+      <c r="B14" s="6"/>
+      <c r="C14" s="5">
         <v>2</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D14" s="6"/>
+      <c r="E14" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="F14" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="G14" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G13" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I13" s="10" t="s">
+      <c r="H14" s="12"/>
+      <c r="I14" s="12" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="14.25">
-      <c r="A14" s="7">
-        <v>8</v>
-      </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="7">
+    <row r="15" spans="1:9" ht="15">
+      <c r="A15" s="5">
+        <v>9</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="5">
         <v>2</v>
       </c>
-      <c r="D14" s="8"/>
-      <c r="E14" s="11" t="s">
+      <c r="D15" s="6"/>
+      <c r="E15" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F15" s="6"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="15">
+      <c r="A16" s="5">
+        <v>10</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="5">
+        <v>2</v>
+      </c>
+      <c r="D16" s="6"/>
+      <c r="E16" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G14" s="13" t="s">
+      <c r="F16" s="6"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="14.25">
-      <c r="A15" s="7">
-        <v>9</v>
-      </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="7">
-        <v>2</v>
-      </c>
-      <c r="D15" s="8"/>
-      <c r="E15" s="11" t="s">
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="14"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="14"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="14"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="14"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="14"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="14.25">
-      <c r="A16" s="7">
-        <v>10</v>
-      </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="7">
-        <v>2</v>
-      </c>
-      <c r="D16" s="8"/>
-      <c r="E16" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="F16" s="8"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17" s="16"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18" s="16"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19" s="16"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" s="16"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="16"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="24"/>
     </row>
     <row r="24" spans="1:9">
-      <c r="A24" s="21"/>
-      <c r="B24" s="21"/>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="21"/>
+      <c r="A24" s="19"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
     </row>
     <row r="25" spans="1:9">
-      <c r="A25" s="22"/>
-      <c r="B25" s="22"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="22"/>
-    </row>
-    <row r="26" spans="1:9" s="23" customFormat="1"/>
+      <c r="A25" s="20"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="20"/>
+    </row>
+    <row r="26" spans="1:9" s="21" customFormat="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="D2:F4"/>
@@ -1195,7 +1206,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1205,7 +1216,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>